<commit_message>
Mapa de flujo: fusiona INFORMIX + paleta de filtro por dominio
- Re-etiqueta destino_externo 'cadena_pru_gtw' -> 'INFORMIX' (4 DB links
  heterogéneos vía gateway en BDPR11G2) para que se fundan con el nodo
  INFORMIX del flujo DataStage. El alias crudo queda en integracion_dblink
  .host_destino.
- /api/flujo ahora entrega los dominios asignados por BD (vía apps) y el
  catálogo de dominios; el tooltip de cada BD muestra sus dominios.
- Nueva paleta '🧩 Dominios' con checkboxes: filtra a las BD que tienen el
  dominio asignado y los nodos conectados a ellas (Todos/Ninguno). Filtro
  combinado con el peso del flujo; usa flags hidden (conserva posiciones).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-05.xlsx
+++ b/client/public/artefactos/ADI-05.xlsx
@@ -3645,7 +3645,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>cadena_pru_gtw</t>
+          <t>INFORMIX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>cadena_pru_gtw</t>
+          <t>INFORMIX</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>cadena_pru_gtw</t>
+          <t>INFORMIX</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>cadena_pru_gtw</t>
+          <t>INFORMIX</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>

</xml_diff>